<commit_message>
Add song reference summaries and current-song research guidance
</commit_message>
<xml_diff>
--- a/资料/资料目录.xlsx
+++ b/资料/资料目录.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>授课日期列记录原稿日期</t>
+          <t>授课日期列记录原稿日期；选歌参考：手语课。情感告别题材，以我、你、朋友之间的叙述与对话推进，副歌重复。可参照否定、条件句、情绪表达及人物指向。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -493,7 +493,7 @@
       <c r="F3" s="11" t="str"/>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>讲义标注日期，授课或发布性质待确认</t>
+          <t>讲义标注日期，授课或发布性质待确认；选歌参考：手语课。成长与陪伴题材，海、道路、路口等意象与抽象心境交织，多分句且副歌反复。可参照比喻具体化、句群拆分和重复动作。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -525,7 +525,7 @@
       <c r="F4" s="10" t="str"/>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>日期据讲义署名</t>
+          <t>日期据讲义署名；选歌参考：手语课。漂泊与故乡题材，第三人称叙事穿插第一人称提问，跨越城市、草原、列车等场景。可参照长修饰句重组、人物视角转换及空间移动。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -557,7 +557,7 @@
       <c r="F5" s="11" t="str"/>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>日期为已确认授课日</t>
+          <t>日期为已确认授课日；选歌参考：手语课。理想与自由题材，雪、风雨、雾等画面承载心理感受，副歌反复。讲义并列呈现字面与内涵取舍，可参照意象处理、否定疑问和抽象表达。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -589,7 +589,7 @@
       <c r="F6" s="10" t="str"/>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>日期为已确认授课日</t>
+          <t>日期为已确认授课日；选歌参考：手语课。自由、平等与抗争题材，由人物生命经历转向群体愿望，副歌反复。讲义呈现不同转写方案，可参照象征意象、抽象概念和语义取舍。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -621,7 +621,7 @@
       <c r="F7" s="11" t="str"/>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>日期为已确认授课日</t>
+          <t>日期为已确认授课日；选歌参考：手语课。怀念与离别题材，星、摇椅、落叶、声音等画面连接对逝者的想象，叙述中穿插呼告和疑问。可参照人物回指、动作方向及情绪与场景转换。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -717,7 +717,7 @@
       <c r="F10" s="10" t="str"/>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>日期据讲义署名</t>
+          <t>日期据讲义署名；选歌参考：手语课。日常生活与喜爱题材，以“我喜欢”串联季节、场所、人物和物件，句式重复而画面频繁切换。可参照列举、数量、位置关系、类标记及专名指拼。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -753,7 +753,7 @@
       <c r="F11" s="11" t="str"/>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>讲义标注日期；当前B版</t>
+          <t>讲义标注日期；当前B版；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -779,7 +779,7 @@
       <c r="F12" s="10" t="str"/>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>秘鲁手语参考手册</t>
+          <t>秘鲁手语参考手册；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -805,7 +805,7 @@
       <c r="F13" s="11" t="str"/>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>四修组长批阅，保留原生批注</t>
+          <t>四修组长批阅，保留原生批注；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -831,7 +831,7 @@
       <c r="F14" s="10" t="str"/>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>早期智能体稿，含协作批注</t>
+          <t>早期智能体稿，含协作批注；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -857,7 +857,7 @@
       <c r="F15" s="11" t="str"/>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>早期智能体稿，含协作批注</t>
+          <t>早期智能体稿，含协作批注；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -883,7 +883,7 @@
       <c r="F16" s="10" t="str"/>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>制作过程稿</t>
+          <t>制作过程稿；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -909,7 +909,7 @@
       <c r="F17" s="11" t="str"/>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>制作过程稿</t>
+          <t>制作过程稿；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -935,7 +935,7 @@
       <c r="F18" s="10" t="str"/>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>制作过程稿</t>
+          <t>制作过程稿；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -961,7 +961,7 @@
       <c r="F19" s="11" t="str"/>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>制作过程稿</t>
+          <t>制作过程稿；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="F20" s="10" t="str"/>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>制作过程稿</t>
+          <t>制作过程稿；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1013,7 +1013,7 @@
       <c r="F21" s="11" t="str"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>教师备注稿；当前主要参照为B版</t>
+          <t>教师备注稿；当前主要参照为B版；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -1039,7 +1039,7 @@
       <c r="F22" s="10" t="str"/>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>教师备注稿；当前主要参照为B版</t>
+          <t>教师备注稿；当前主要参照为B版；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1065,7 +1065,7 @@
       <c r="F23" s="11" t="str"/>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>打印稿；当前主要参照为B版</t>
+          <t>打印稿；当前主要参照为B版；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -1091,7 +1091,7 @@
       <c r="F24" s="10" t="str"/>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>早期智能体稿，含协作批注</t>
+          <t>早期智能体稿，含协作批注；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -1117,7 +1117,7 @@
       <c r="F25" s="11" t="str"/>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>早期智能体稿，含协作批注</t>
+          <t>早期智能体稿，含协作批注；选歌参考：手语课。古文明、祭典与文化交流题材，主歌铺陈文物和场景，过渡含选择疑问，副歌重复并穿插接句。可参照文化词汇、抽象意象具体化及主句与接句组织。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -1177,7 +1177,7 @@
       <c r="F27" s="11" t="str"/>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>带批注讲义；原文署名2026.4.11</t>
+          <t>带批注讲义；原文署名2026.4.11；选歌参考：手语课。以两只毛毛虫化蝶叙述相伴、分离与成长，中英对照并有重复副歌。可参照双主体空间、蛹的内外关系、类标记和成长隐喻；须区分语言版本。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -1207,7 +1207,7 @@
       <c r="F28" s="10" t="str"/>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>最终版本（手语老师确认）；3.0ver；原文署名2025.3.22；选择参照材料时优先使用本稿</t>
+          <t>最终版本（手语老师确认）；3.0ver；原文署名2025.3.22；选择参照材料时优先使用本稿；选歌参考：手语课。日常幸福与自我陪伴题材，路口、云、狗、树叶等具体画面带有拟人和比喻，短句与重复段较多。可参照日常词汇、拟人画面和情绪表达。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -1237,7 +1237,7 @@
       <c r="F29" s="11" t="str"/>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>较早版本，供比较修改；最终版本为Re Re Re手语课讲义 小美满 3.0ver.docx</t>
+          <t>较早版本，供比较修改；最终版本为Re Re Re手语课讲义 小美满 3.0ver.docx；选歌参考：手语课。日常幸福与自我陪伴题材，路口、云、狗、树叶等具体画面带有拟人和比喻，短句与重复段较多。可参照日常词汇、拟人画面和情绪表达。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -1263,7 +1263,7 @@
       <c r="F30" s="10" t="str"/>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>初稿（改）2.0，带批注；与已有定稿并存</t>
+          <t>初稿（改）2.0，带批注；与已有定稿并存；选歌参考：手语课。怀念与离别题材，星、摇椅、落叶、声音等画面连接对逝者的想象，叙述中穿插呼告和疑问。可参照人物回指、动作方向及情绪与场景转换。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -1293,7 +1293,7 @@
       <c r="F31" s="11" t="str"/>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>终稿PDF，6页；正文署名2026.4.11；不以文件修改时间判定授课日期</t>
+          <t>终稿PDF，6页；正文署名2026.4.11；不以文件修改时间判定授课日期；选歌参考：手语课。以两只毛毛虫化蝶叙述相伴、分离与成长，中英对照并有重复副歌。可参照双主体空间、蛹的内外关系、类标记和成长隐喻；须区分语言版本。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -1323,7 +1323,7 @@
       <c r="F32" s="10" t="str"/>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>三改PDF，6页；正文署名2026.4.11；不以文件修改时间判定授课日期</t>
+          <t>三改PDF，6页；正文署名2026.4.11；不以文件修改时间判定授课日期；选歌参考：手语课。以两只毛毛虫化蝶叙述相伴、分离与成长，中英对照并有重复副歌。可参照双主体空间、蛹的内外关系、类标记和成长隐喻；须区分语言版本。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -1353,7 +1353,7 @@
       <c r="F33" s="11" t="str"/>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>二改PDF，6页；正文署名2026.4.11；不以文件修改时间判定授课日期</t>
+          <t>二改PDF，6页；正文署名2026.4.11；不以文件修改时间判定授课日期；选歌参考：手语课。以两只毛毛虫化蝶叙述相伴、分离与成长，中英对照并有重复副歌。可参照双主体空间、蛹的内外关系、类标记和成长隐喻；须区分语言版本。节奏须结合音频核对。</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Fit song reference notes within catalog rows
</commit_message>
<xml_diff>
--- a/资料/资料目录.xlsx
+++ b/资料/资料目录.xlsx
@@ -432,7 +432,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="76" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
           <t>其实讲义editby二萌.docx</t>
@@ -470,7 +470,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="76" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>RE永远都会在 讲义 2.0ver (1).docx</t>
@@ -502,7 +502,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="76" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>历历万乡.pdf</t>
@@ -534,7 +534,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="76" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>海阔天空.docx</t>
@@ -566,7 +566,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="76" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>光辉岁月讲义 (1).docx</t>
@@ -598,7 +598,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
+    <row r="7" ht="76" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>《暮色回响》手语讲义定稿（已校）.docx</t>
@@ -694,7 +694,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
+    <row r="10" ht="76" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>我喜欢Ver1editby二萌.pdf</t>
@@ -726,7 +726,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
+    <row r="11" ht="93" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>太阳升起的舞蹈_讲义版_B版.docx</t>
@@ -762,7 +762,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="42" customHeight="1">
+    <row r="12" ht="93" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Manual de lenguaje de señas peruanas.pdf</t>
@@ -788,7 +788,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="42" customHeight="1">
+    <row r="13" ht="93" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>RE太阳升起的舞蹈_教学整理版_四修.docx</t>
@@ -814,7 +814,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="42" customHeight="1">
+    <row r="14" ht="93" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>太阳升起的舞蹈_手语翻译_拓宽版.docx</t>
@@ -840,7 +840,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="42" customHeight="1">
+    <row r="15" ht="93" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>太阳升起的舞蹈_手语翻译_纯译版.docx</t>
@@ -866,7 +866,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1">
+    <row r="16" ht="76" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>太阳升起的舞蹈_教学整理版_三修.docx</t>
@@ -892,7 +892,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="42" customHeight="1">
+    <row r="17" ht="76" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>太阳升起的舞蹈_教学整理版_二修.docx</t>
@@ -918,7 +918,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1">
+    <row r="18" ht="76" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>太阳升起的舞蹈_教学整理版_修订.docx</t>
@@ -944,7 +944,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="42" customHeight="1">
+    <row r="19" ht="76" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>太阳升起的舞蹈_教学整理版_四修.docx</t>
@@ -970,7 +970,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="42" customHeight="1">
+    <row r="20" ht="76" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>太阳升起的舞蹈_教学整理版_贴图工作稿.docx</t>
@@ -996,7 +996,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="42" customHeight="1">
+    <row r="21" ht="93" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>太阳升起的舞蹈_老师注释版_二萌修后_A版.docx</t>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="42" customHeight="1">
+    <row r="22" ht="93" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>太阳升起的舞蹈_老师注释版_组长修后_B版.docx</t>
@@ -1048,7 +1048,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="42" customHeight="1">
+    <row r="23" ht="93" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>太阳升起的舞蹈_讲义版_A版.docx</t>
@@ -1074,7 +1074,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="42" customHeight="1">
+    <row r="24" ht="93" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>输出目录_太阳升起的舞蹈_手语翻译_拓宽版.docx</t>
@@ -1100,7 +1100,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="42" customHeight="1">
+    <row r="25" ht="93" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>输出目录_太阳升起的舞蹈_手语翻译_纯译版.docx</t>
@@ -1156,7 +1156,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="42" customHeight="1">
+    <row r="27" ht="93" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>RETwo Oruguitas.docx</t>
@@ -1186,7 +1186,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="42" customHeight="1">
+    <row r="28" ht="110" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Re Re Re手语课讲义 小美满 3.0ver.docx</t>
@@ -1216,7 +1216,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="42" customHeight="1">
+    <row r="29" ht="110" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Re Re手语课讲义 小美满 3.0ver.docx</t>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="42" customHeight="1">
+    <row r="30" ht="93" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>RE《暮色回响》手语讲义初稿（改）2.0.docx</t>
@@ -1272,7 +1272,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="42" customHeight="1">
+    <row r="31" ht="93" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Two Oruguitas - 联星&amp;八月 - 终稿.pdf</t>
@@ -1302,7 +1302,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="42" customHeight="1">
+    <row r="32" ht="93" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Two Oruguitas - 三改.pdf</t>
@@ -1332,7 +1332,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="42" customHeight="1">
+    <row r="33" ht="93" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
           <t>Two Oruguitas - 二改.pdf</t>

</xml_diff>